<commit_message>
Making Fixes In Ui and Credits System
</commit_message>
<xml_diff>
--- a/examples/Company_Data/financials_bundle.xlsx
+++ b/examples/Company_Data/financials_bundle.xlsx
@@ -490,7 +490,7 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>14.95</v>
+        <v>17747116.07</v>
       </c>
       <c r="E2" t="n">
         <v>16.54</v>
@@ -519,7 +519,7 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>11.64</v>
+        <v>13815307.89</v>
       </c>
       <c r="E3" t="n">
         <v>14.9</v>
@@ -548,7 +548,7 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>12.96</v>
+        <v>15390801.88</v>
       </c>
       <c r="E4" t="n">
         <v>14.11</v>
@@ -577,7 +577,7 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>27.8</v>
+        <v>33011143.96</v>
       </c>
       <c r="E5" t="n">
         <v>14.9</v>
@@ -606,7 +606,7 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>17.28</v>
+        <v>20511921.02</v>
       </c>
       <c r="E6" t="n">
         <v>15.39</v>
@@ -635,7 +635,7 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>15.37</v>
+        <v>18250059.47</v>
       </c>
       <c r="E7" t="n">
         <v>13.32</v>

</xml_diff>